<commit_message>
fix(html): modal print button and font size issue
</commit_message>
<xml_diff>
--- a/.source/kb023_information.xlsx
+++ b/.source/kb023_information.xlsx
@@ -968,19 +968,15 @@
       <c r="A7" s="10" t="n">
         <v>46059</v>
       </c>
-      <c r="B7" s="0" t="n"/>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>비동의</t>
-        </is>
-      </c>
+      <c r="B7" s="0" t="inlineStr"/>
+      <c r="C7" s="0" t="inlineStr"/>
       <c r="D7" s="0" t="inlineStr">
         <is>
           <t>일반</t>
         </is>
       </c>
-      <c r="E7" s="0" t="n"/>
-      <c r="F7" s="0" t="n"/>
+      <c r="E7" s="0" t="inlineStr"/>
+      <c r="F7" s="0" t="inlineStr"/>
       <c r="G7" s="0" t="inlineStr">
         <is>
           <t>나종상</t>
@@ -993,7 +989,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>010-3341-2789</t>
+          <t>003-341-2789</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
@@ -1006,14 +1002,10 @@
           <t>서울 관악 삼모더프라임타워 2405호</t>
         </is>
       </c>
-      <c r="L7" s="0" t="inlineStr">
-        <is>
-          <t>나종상</t>
-        </is>
-      </c>
+      <c r="L7" s="0" t="inlineStr"/>
       <c r="M7" s="0" t="inlineStr">
         <is>
-          <t>751208-1654415</t>
+          <t>800801-1234567</t>
         </is>
       </c>
       <c r="N7" s="0" t="inlineStr">

</xml_diff>